<commit_message>
Make tutorial runs optional after the first
</commit_message>
<xml_diff>
--- a/tutorial/scoring/ref13-scoring-template.xlsx
+++ b/tutorial/scoring/ref13-scoring-template.xlsx
@@ -34,7 +34,7 @@
     <t xml:space="preserve">Paste one model answer for ref13 into a Run tab. The workbook compares its 42 fields with the six-row benchmark.</t>
   </si>
   <si>
-    <t xml:space="preserve">HOW TO USE IT</t>
+    <t xml:space="preserve">HOW TO USE IT — ONE RUN IS ENOUGH</t>
   </si>
   <si>
     <t xml:space="preserve">1.  Go to the 'Run 1' tab.</t>
@@ -55,10 +55,10 @@
     <t xml:space="preserve">     enter a corrected whole-row score from 0 to 7 in the yellow Your /7 cell.</t>
   </si>
   <si>
-    <t xml:space="preserve">6.  Quick path: complete Run 1. Full path: repeat in fresh chats for Runs 2–5.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7.  Scoreboard shows accuracy for completed runs. Consistency appears after all 5 runs.</t>
+    <t xml:space="preserve">6.  One run is enough. Ignore Run 2–Run 5 unless you choose to repeat later.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.  Open Scoreboard for Run 1 accuracy. Repeat summaries are optional.</t>
   </si>
   <si>
     <t xml:space="preserve">GOOD TO KNOW</t>
@@ -73,7 +73,7 @@
     <t xml:space="preserve">•  Ignore extra high-affinity K1 rows. Record their count in the yellow box if useful.</t>
   </si>
   <si>
-    <t xml:space="preserve">•  The Scoreboard says Incomplete until every blue cell in a run is filled.</t>
+    <t xml:space="preserve">•  Scoreboard says Incomplete until every blue cell in a run is filled.</t>
   </si>
   <si>
     <t xml:space="preserve">•  If the answer is not one clean table, use prompts/2-normalizer-prompt.md first.</t>
@@ -229,7 +229,7 @@
     <t xml:space="preserve">Scoreboard</t>
   </si>
   <si>
-    <t xml:space="preserve">Accuracy against the benchmark (how correct)</t>
+    <t xml:space="preserve">Accuracy (one run is enough; additional runs are optional)</t>
   </si>
   <si>
     <t xml:space="preserve">Run</t>
@@ -256,13 +256,13 @@
     <t xml:space="preserve">Run 5</t>
   </si>
   <si>
-    <t xml:space="preserve">Average (completed runs)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Consistency across runs (how repeatable)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Of the 42 fields, the share where all five completed runs gave the same normalized value.</t>
+    <t xml:space="preserve">Optional average (completed runs)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional consistency across repeated runs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">If all five optional runs are complete, this shows the share of fields where every run gave the same normalized value.</t>
   </si>
   <si>
     <t xml:space="preserve">Consistent fields:</t>
@@ -274,7 +274,7 @@
     <t xml:space="preserve">Consistency %:</t>
   </si>
   <si>
-    <t xml:space="preserve">(Consistency appears only after all five runs are complete.)</t>
+    <t xml:space="preserve">(Optional: consistency appears only after all five Run tabs are complete.)</t>
   </si>
 </sst>
 </file>
@@ -433,7 +433,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="33">
+  <cellStyleXfs count="39">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -459,11 +459,15 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="166" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="167" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="168" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="169" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="170" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="170" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="171" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="172" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="172" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
@@ -477,6 +481,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="173" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="173" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="173" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
@@ -485,84 +494,84 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="29" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="33" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="29" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="33" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="29" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="33" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="29" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="33" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="29" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="33" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="0" xfId="29" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="0" xfId="33" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="29" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="33" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="0" xfId="29" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="5" borderId="0" xfId="33" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="29" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="33" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="29" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="33" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="6" borderId="1" xfId="29" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="1" xfId="33" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="7" borderId="1" xfId="29" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="7" borderId="1" xfId="33" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="29" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="33" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="8" borderId="1" xfId="29" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="8" borderId="1" xfId="33" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="29" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="33" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="7" fillId="0" borderId="0" xfId="29" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="173" fontId="7" fillId="0" borderId="0" xfId="33" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="29" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="33" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="5" fillId="0" borderId="1" xfId="29" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="173" fontId="5" fillId="0" borderId="1" xfId="33" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="7" fillId="0" borderId="0" xfId="29" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="173" fontId="7" fillId="0" borderId="0" xfId="33" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
-  <cellStyles count="19">
+  <cellStyles count="25">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Comma" xfId="15" builtinId="3"/>
     <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
@@ -571,17 +580,23 @@
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
     <cellStyle name="Comma" xfId="20"/>
     <cellStyle name="Comma 1" xfId="21"/>
-    <cellStyle name="Comma [0]" xfId="22"/>
-    <cellStyle name="Comma [0] 2" xfId="23"/>
-    <cellStyle name="Currency" xfId="24"/>
-    <cellStyle name="Currency 3" xfId="25"/>
-    <cellStyle name="Currency [0]" xfId="26"/>
-    <cellStyle name="Currency [0] 4" xfId="27"/>
-    <cellStyle name="Normal" xfId="28"/>
-    <cellStyle name="Normal 1" xfId="29"/>
-    <cellStyle name="Normal 5" xfId="30"/>
-    <cellStyle name="Percent" xfId="31"/>
-    <cellStyle name="Percent 6" xfId="32"/>
+    <cellStyle name="Comma 2" xfId="22"/>
+    <cellStyle name="Comma [0]" xfId="23"/>
+    <cellStyle name="Comma [0] 2" xfId="24"/>
+    <cellStyle name="Comma [0] 3" xfId="25"/>
+    <cellStyle name="Currency" xfId="26"/>
+    <cellStyle name="Currency 3" xfId="27"/>
+    <cellStyle name="Currency 4" xfId="28"/>
+    <cellStyle name="Currency [0]" xfId="29"/>
+    <cellStyle name="Currency [0] 4" xfId="30"/>
+    <cellStyle name="Currency [0] 5" xfId="31"/>
+    <cellStyle name="Normal" xfId="32"/>
+    <cellStyle name="Normal 1" xfId="33"/>
+    <cellStyle name="Normal 5" xfId="34"/>
+    <cellStyle name="Normal 6" xfId="35"/>
+    <cellStyle name="Percent" xfId="36"/>
+    <cellStyle name="Percent 6" xfId="37"/>
+    <cellStyle name="Percent 7" xfId="38"/>
   </cellStyles>
   <colors>
     <indexedColors>

</xml_diff>

<commit_message>
Make one tutorial run the default (#2)
Make one extraction per lab the complete tutorial flow while keeping additional runs optional. Preserve all four research prompt files unchanged.
</commit_message>
<xml_diff>
--- a/tutorial/scoring/ref13-scoring-template.xlsx
+++ b/tutorial/scoring/ref13-scoring-template.xlsx
@@ -34,7 +34,7 @@
     <t xml:space="preserve">Paste one model answer for ref13 into a Run tab. The workbook compares its 42 fields with the six-row benchmark.</t>
   </si>
   <si>
-    <t xml:space="preserve">HOW TO USE IT</t>
+    <t xml:space="preserve">HOW TO USE IT — ONE RUN IS ENOUGH</t>
   </si>
   <si>
     <t xml:space="preserve">1.  Go to the 'Run 1' tab.</t>
@@ -55,10 +55,10 @@
     <t xml:space="preserve">     enter a corrected whole-row score from 0 to 7 in the yellow Your /7 cell.</t>
   </si>
   <si>
-    <t xml:space="preserve">6.  Quick path: complete Run 1. Full path: repeat in fresh chats for Runs 2–5.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7.  Scoreboard shows accuracy for completed runs. Consistency appears after all 5 runs.</t>
+    <t xml:space="preserve">6.  One run is enough. Ignore Run 2–Run 5 unless you choose to repeat later.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.  Open Scoreboard for Run 1 accuracy. Repeat summaries are optional.</t>
   </si>
   <si>
     <t xml:space="preserve">GOOD TO KNOW</t>
@@ -73,7 +73,7 @@
     <t xml:space="preserve">•  Ignore extra high-affinity K1 rows. Record their count in the yellow box if useful.</t>
   </si>
   <si>
-    <t xml:space="preserve">•  The Scoreboard says Incomplete until every blue cell in a run is filled.</t>
+    <t xml:space="preserve">•  Scoreboard says Incomplete until every blue cell in a run is filled.</t>
   </si>
   <si>
     <t xml:space="preserve">•  If the answer is not one clean table, use prompts/2-normalizer-prompt.md first.</t>
@@ -229,7 +229,7 @@
     <t xml:space="preserve">Scoreboard</t>
   </si>
   <si>
-    <t xml:space="preserve">Accuracy against the benchmark (how correct)</t>
+    <t xml:space="preserve">Accuracy (one run is enough; additional runs are optional)</t>
   </si>
   <si>
     <t xml:space="preserve">Run</t>
@@ -256,13 +256,13 @@
     <t xml:space="preserve">Run 5</t>
   </si>
   <si>
-    <t xml:space="preserve">Average (completed runs)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Consistency across runs (how repeatable)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Of the 42 fields, the share where all five completed runs gave the same normalized value.</t>
+    <t xml:space="preserve">Optional average (completed runs)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional consistency across repeated runs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">If all five optional runs are complete, this shows the share of fields where every run gave the same normalized value.</t>
   </si>
   <si>
     <t xml:space="preserve">Consistent fields:</t>
@@ -274,7 +274,7 @@
     <t xml:space="preserve">Consistency %:</t>
   </si>
   <si>
-    <t xml:space="preserve">(Consistency appears only after all five runs are complete.)</t>
+    <t xml:space="preserve">(Optional: consistency appears only after all five Run tabs are complete.)</t>
   </si>
 </sst>
 </file>
@@ -433,7 +433,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="33">
+  <cellStyleXfs count="39">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -459,11 +459,15 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="166" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="167" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="168" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="169" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="170" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="170" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="171" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="172" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="172" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
@@ -477,6 +481,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="173" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="173" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="173" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
@@ -485,84 +494,84 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="29" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="33" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="29" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="33" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="29" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="33" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="29" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="33" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="29" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="33" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="0" xfId="29" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="0" xfId="33" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="29" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="33" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="0" xfId="29" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="5" borderId="0" xfId="33" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="29" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="33" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="29" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="33" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="6" borderId="1" xfId="29" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="1" xfId="33" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="7" borderId="1" xfId="29" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="7" borderId="1" xfId="33" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="29" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="33" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="8" borderId="1" xfId="29" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="8" borderId="1" xfId="33" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="29" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="33" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="7" fillId="0" borderId="0" xfId="29" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="173" fontId="7" fillId="0" borderId="0" xfId="33" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="29" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="33" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="5" fillId="0" borderId="1" xfId="29" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="173" fontId="5" fillId="0" borderId="1" xfId="33" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="7" fillId="0" borderId="0" xfId="29" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="173" fontId="7" fillId="0" borderId="0" xfId="33" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
-  <cellStyles count="19">
+  <cellStyles count="25">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Comma" xfId="15" builtinId="3"/>
     <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
@@ -571,17 +580,23 @@
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
     <cellStyle name="Comma" xfId="20"/>
     <cellStyle name="Comma 1" xfId="21"/>
-    <cellStyle name="Comma [0]" xfId="22"/>
-    <cellStyle name="Comma [0] 2" xfId="23"/>
-    <cellStyle name="Currency" xfId="24"/>
-    <cellStyle name="Currency 3" xfId="25"/>
-    <cellStyle name="Currency [0]" xfId="26"/>
-    <cellStyle name="Currency [0] 4" xfId="27"/>
-    <cellStyle name="Normal" xfId="28"/>
-    <cellStyle name="Normal 1" xfId="29"/>
-    <cellStyle name="Normal 5" xfId="30"/>
-    <cellStyle name="Percent" xfId="31"/>
-    <cellStyle name="Percent 6" xfId="32"/>
+    <cellStyle name="Comma 2" xfId="22"/>
+    <cellStyle name="Comma [0]" xfId="23"/>
+    <cellStyle name="Comma [0] 2" xfId="24"/>
+    <cellStyle name="Comma [0] 3" xfId="25"/>
+    <cellStyle name="Currency" xfId="26"/>
+    <cellStyle name="Currency 3" xfId="27"/>
+    <cellStyle name="Currency 4" xfId="28"/>
+    <cellStyle name="Currency [0]" xfId="29"/>
+    <cellStyle name="Currency [0] 4" xfId="30"/>
+    <cellStyle name="Currency [0] 5" xfId="31"/>
+    <cellStyle name="Normal" xfId="32"/>
+    <cellStyle name="Normal 1" xfId="33"/>
+    <cellStyle name="Normal 5" xfId="34"/>
+    <cellStyle name="Normal 6" xfId="35"/>
+    <cellStyle name="Percent" xfId="36"/>
+    <cellStyle name="Percent 6" xfId="37"/>
+    <cellStyle name="Percent 7" xfId="38"/>
   </cellStyles>
   <colors>
     <indexedColors>

</xml_diff>